<commit_message>
New Implementation of Faster Parsing
</commit_message>
<xml_diff>
--- a/src/test/resources/skipHiddenTestData.xlsx
+++ b/src/test/resources/skipHiddenTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bradjacobs/git/bradjacobs/excel-to-csv/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CFF4CEF-012A-6D4E-9123-F4CC71630269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8FF31F3-FAB4-CD47-9C4B-172DC352964F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" firstSheet="9" activeTab="12" xr2:uid="{F0E37EA6-B81C-114C-AD9D-8AE6FA3EF7BF}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" firstSheet="16" activeTab="21" xr2:uid="{F0E37EA6-B81C-114C-AD9D-8AE6FA3EF7BF}"/>
   </bookViews>
   <sheets>
     <sheet name="BaseCase_Data" sheetId="1" r:id="rId1"/>
@@ -29,6 +29,12 @@
     <sheet name="LastValueInvisible_Expected" sheetId="14" r:id="rId14"/>
     <sheet name="LongestRowInvisible_Data" sheetId="15" r:id="rId15"/>
     <sheet name="LongestRowInvisible_Expected" sheetId="16" r:id="rId16"/>
+    <sheet name="MiddleBlankRows_Data" sheetId="17" r:id="rId17"/>
+    <sheet name="MiddleBlankRows_Expected" sheetId="18" r:id="rId18"/>
+    <sheet name="MiddleBlankColumns_Data" sheetId="20" r:id="rId19"/>
+    <sheet name="MiddleBlankColumns_Expected" sheetId="21" r:id="rId20"/>
+    <sheet name="LastInvisible_Data" sheetId="22" r:id="rId21"/>
+    <sheet name="LastInvisible_Expected" sheetId="23" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="62">
   <si>
     <t>dd</t>
   </si>
@@ -222,6 +228,21 @@
   </si>
   <si>
     <t>ddd</t>
+  </si>
+  <si>
+    <t>aaa</t>
+  </si>
+  <si>
+    <t>bbb</t>
+  </si>
+  <si>
+    <t>ccc</t>
+  </si>
+  <si>
+    <t>yyy</t>
+  </si>
+  <si>
+    <t>zzz</t>
   </si>
 </sst>
 </file>
@@ -797,7 +818,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D42D809-2413-7D42-9528-29078949896B}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.1640625" customWidth="1"/>
@@ -932,6 +953,91 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD097AA0-5C13-4043-BDF1-006D5C80261E}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:2" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="1:2" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3416C67B-AEC0-864E-B663-478C9C2764FF}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{870638FC-E3D2-EA4F-BE7C-542AE36A7465}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="5" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{453B851B-2721-4E4B-B8B9-D77A87CF85CE}">
   <dimension ref="A1:B4"/>
@@ -956,6 +1062,76 @@
       </c>
       <c r="B4" t="s">
         <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F5FA91-6D56-2F41-9D05-97C28C5B7749}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2D38582-62F2-604F-B6D0-843142BB203A}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="0" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C31D898E-E30A-754F-B984-2FC77D02F868}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
interim step refactor: remove visibilty reference from the SheetDataHandler class
</commit_message>
<xml_diff>
--- a/src/test/resources/skipHiddenTestData.xlsx
+++ b/src/test/resources/skipHiddenTestData.xlsx
@@ -8,33 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bradjacobs/git/bradjacobs/excel-to-csv/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8FF31F3-FAB4-CD47-9C4B-172DC352964F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4690FF-F047-4547-A1C5-84235C853EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" firstSheet="16" activeTab="21" xr2:uid="{F0E37EA6-B81C-114C-AD9D-8AE6FA3EF7BF}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="4" xr2:uid="{F0E37EA6-B81C-114C-AD9D-8AE6FA3EF7BF}"/>
   </bookViews>
   <sheets>
     <sheet name="BaseCase_Data" sheetId="1" r:id="rId1"/>
     <sheet name="BaseCase_Expected" sheetId="2" r:id="rId2"/>
-    <sheet name="LastColumn_Data" sheetId="3" r:id="rId3"/>
-    <sheet name="LastColumn_Expected" sheetId="4" r:id="rId4"/>
-    <sheet name="FirstLastRow_Data" sheetId="5" r:id="rId5"/>
-    <sheet name="FirstLastRow_Expected" sheetId="6" r:id="rId6"/>
-    <sheet name="AllColumnHidden_Data" sheetId="7" r:id="rId7"/>
-    <sheet name="AllColumnHidden_Expected" sheetId="8" r:id="rId8"/>
-    <sheet name="FirstLastColumn_Data" sheetId="9" r:id="rId9"/>
-    <sheet name="FirstLastColumn_Expected" sheetId="10" r:id="rId10"/>
-    <sheet name="Multi_Data" sheetId="11" r:id="rId11"/>
-    <sheet name="Multi_Expected" sheetId="12" r:id="rId12"/>
-    <sheet name="LastValueInvisible_Data" sheetId="13" r:id="rId13"/>
-    <sheet name="LastValueInvisible_Expected" sheetId="14" r:id="rId14"/>
-    <sheet name="LongestRowInvisible_Data" sheetId="15" r:id="rId15"/>
-    <sheet name="LongestRowInvisible_Expected" sheetId="16" r:id="rId16"/>
-    <sheet name="MiddleBlankRows_Data" sheetId="17" r:id="rId17"/>
-    <sheet name="MiddleBlankRows_Expected" sheetId="18" r:id="rId18"/>
-    <sheet name="MiddleBlankColumns_Data" sheetId="20" r:id="rId19"/>
-    <sheet name="MiddleBlankColumns_Expected" sheetId="21" r:id="rId20"/>
-    <sheet name="LastInvisible_Data" sheetId="22" r:id="rId21"/>
-    <sheet name="LastInvisible_Expected" sheetId="23" r:id="rId22"/>
+    <sheet name="SingleHiddenRow_Data" sheetId="25" r:id="rId3"/>
+    <sheet name="SingleHiddenRow_Expected" sheetId="24" r:id="rId4"/>
+    <sheet name="SingleHiddenColumn_Data" sheetId="27" r:id="rId5"/>
+    <sheet name="SingleHiddenColumn_Expected" sheetId="26" r:id="rId6"/>
+    <sheet name="LastColumn_Data" sheetId="3" r:id="rId7"/>
+    <sheet name="LastColumn_Expected" sheetId="4" r:id="rId8"/>
+    <sheet name="FirstLastRow_Data" sheetId="5" r:id="rId9"/>
+    <sheet name="FirstLastRow_Expected" sheetId="6" r:id="rId10"/>
+    <sheet name="AllColumnHidden_Data" sheetId="7" r:id="rId11"/>
+    <sheet name="AllColumnHidden_Expected" sheetId="8" r:id="rId12"/>
+    <sheet name="FirstLastColumn_Data" sheetId="9" r:id="rId13"/>
+    <sheet name="FirstLastColumn_Expected" sheetId="10" r:id="rId14"/>
+    <sheet name="Multi_Data" sheetId="11" r:id="rId15"/>
+    <sheet name="Multi_Expected" sheetId="12" r:id="rId16"/>
+    <sheet name="LastValueInvisible_Data" sheetId="13" r:id="rId17"/>
+    <sheet name="LastValueInvisible_Expected" sheetId="14" r:id="rId18"/>
+    <sheet name="LongestRowInvisible_Data" sheetId="15" r:id="rId19"/>
+    <sheet name="LongestRowInvisible_Expected" sheetId="16" r:id="rId20"/>
+    <sheet name="MiddleBlankRows_Data" sheetId="17" r:id="rId21"/>
+    <sheet name="MiddleBlankRows_Expected" sheetId="18" r:id="rId22"/>
+    <sheet name="MiddleBlankColumns_Data" sheetId="20" r:id="rId23"/>
+    <sheet name="MiddleBlankColumns_Expected" sheetId="21" r:id="rId24"/>
+    <sheet name="LastInvisible_Data" sheetId="22" r:id="rId25"/>
+    <sheet name="LastInvisible_Expected" sheetId="23" r:id="rId26"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="64">
   <si>
     <t>dd</t>
   </si>
@@ -243,6 +247,12 @@
   </si>
   <si>
     <t>zzz</t>
+  </si>
+  <si>
+    <t>eee</t>
+  </si>
+  <si>
+    <t>fff</t>
   </si>
 </sst>
 </file>
@@ -677,6 +687,99 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDF8D2F8-2790-474D-812E-AB3A3917770A}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CC0E83-C807-B643-BCAE-31CED9BEE75A}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="10.83203125" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7571C826-D0E5-C441-A8DD-7EE05C8C6CE6}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C821FD3-AB01-2F4B-9E43-FE867B4E795E}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4782EB7B-497F-CB49-AC44-66541F555E13}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -691,7 +794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7542B299-0860-9D4E-BA17-70A5DA5AA3FF}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -790,7 +893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42594AB4-EFE5-204B-81AD-38E0779347C9}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -816,7 +919,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D42D809-2413-7D42-9528-29078949896B}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -849,7 +952,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB789F4-B352-C44A-AC05-1E9CB856ADE9}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -875,7 +978,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0685FA5C-3B1B-8B43-A0DE-C31877AC6617}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -924,7 +1027,38 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{453B851B-2721-4E4B-B8B9-D77A87CF85CE}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24EC2481-D362-CE42-910F-8498EA2FA4FC}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -953,7 +1087,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD097AA0-5C13-4043-BDF1-006D5C80261E}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -982,7 +1116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3416C67B-AEC0-864E-B663-478C9C2764FF}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1008,7 +1142,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{870638FC-E3D2-EA4F-BE7C-542AE36A7465}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1038,38 +1172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{453B851B-2721-4E4B-B8B9-D77A87CF85CE}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F5FA91-6D56-2F41-9D05-97C28C5B7749}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1095,7 +1198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2D38582-62F2-604F-B6D0-843142BB203A}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1124,7 +1227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C31D898E-E30A-754F-B984-2FC77D02F868}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1140,6 +1243,127 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5261E835-3C7B-8540-86E0-56BD5E8AF73D}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BA209BC-D001-C84F-A7A3-4CF5790BE342}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9295F5CD-96CE-8B4F-93FA-2B550E947343}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="0" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB302F3-DD94-F946-8644-B37CCADD53D3}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A4D3C3B-C67B-EE48-84CE-DB39EEBE467A}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1177,7 +1401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F13273A8-FCD7-0E4D-8111-34289EC7BF1F}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1205,7 +1429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{894093BD-B389-F34D-8CD3-B45445B09925}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1252,97 +1476,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDF8D2F8-2790-474D-812E-AB3A3917770A}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CC0E83-C807-B643-BCAE-31CED9BEE75A}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="10.83203125" hidden="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7571C826-D0E5-C441-A8DD-7EE05C8C6CE6}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C821FD3-AB01-2F4B-9E43-FE867B4E795E}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" hidden="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
update to use term 'hidden' instead of 'invisible'
</commit_message>
<xml_diff>
--- a/src/test/resources/skipHiddenTestData.xlsx
+++ b/src/test/resources/skipHiddenTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bradjacobs/git/bradjacobs/excel-to-csv/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4690FF-F047-4547-A1C5-84235C853EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E497BA-FBF6-6449-ABF2-DD8858DBCE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="4" xr2:uid="{F0E37EA6-B81C-114C-AD9D-8AE6FA3EF7BF}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" xr2:uid="{F0E37EA6-B81C-114C-AD9D-8AE6FA3EF7BF}"/>
   </bookViews>
   <sheets>
     <sheet name="BaseCase_Data" sheetId="1" r:id="rId1"/>
@@ -29,16 +29,16 @@
     <sheet name="FirstLastColumn_Expected" sheetId="10" r:id="rId14"/>
     <sheet name="Multi_Data" sheetId="11" r:id="rId15"/>
     <sheet name="Multi_Expected" sheetId="12" r:id="rId16"/>
-    <sheet name="LastValueInvisible_Data" sheetId="13" r:id="rId17"/>
-    <sheet name="LastValueInvisible_Expected" sheetId="14" r:id="rId18"/>
-    <sheet name="LongestRowInvisible_Data" sheetId="15" r:id="rId19"/>
-    <sheet name="LongestRowInvisible_Expected" sheetId="16" r:id="rId20"/>
+    <sheet name="LastValueHidden_Data" sheetId="13" r:id="rId17"/>
+    <sheet name="LastValueHidden_Expected" sheetId="14" r:id="rId18"/>
+    <sheet name="LongestRowHidden_Data" sheetId="15" r:id="rId19"/>
+    <sheet name="LongestRowHidden_Expected" sheetId="16" r:id="rId20"/>
     <sheet name="MiddleBlankRows_Data" sheetId="17" r:id="rId21"/>
     <sheet name="MiddleBlankRows_Expected" sheetId="18" r:id="rId22"/>
     <sheet name="MiddleBlankColumns_Data" sheetId="20" r:id="rId23"/>
     <sheet name="MiddleBlankColumns_Expected" sheetId="21" r:id="rId24"/>
-    <sheet name="LastInvisible_Data" sheetId="22" r:id="rId25"/>
-    <sheet name="LastInvisible_Expected" sheetId="23" r:id="rId26"/>
+    <sheet name="LastHidden_Data" sheetId="22" r:id="rId25"/>
+    <sheet name="LastHidden_Expected" sheetId="23" r:id="rId26"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>